<commit_message>
Fill remaining gaps, add item numbers, re-export inventory
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ftyu6Z5XGtgfDh47rmypeJ
</commit_message>
<xml_diff>
--- a/inventory-2026-08-14.xlsx
+++ b/inventory-2026-08-14.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Inventory" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$H$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Inventory'!$A$1:$I$16</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -81,10 +81,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -460,589 +463,648 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H16"/>
+  <dimension ref="A1:I16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="32" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
-    <col width="34" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="26" customWidth="1" min="5" max="5"/>
+    <col width="9" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
     <col width="26" customWidth="1" min="6" max="6"/>
-    <col width="11" customWidth="1" min="7" max="7"/>
-    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="26" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>Item No.</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
           <t>Product Name</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Colour Clarity/Description</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Defects</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Size</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Condition</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>SKU</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Price</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Date Added</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
         <is>
           <t>Skinny Minnie</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr"/>
-      <c r="C2" s="2" t="inlineStr"/>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="C2" s="3" t="inlineStr"/>
+      <c r="D2" s="3" t="inlineStr"/>
+      <c r="E2" s="3" t="inlineStr">
         <is>
           <t>Large Women's</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="F2" s="3" t="inlineStr">
         <is>
           <t>Very good condition</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="G2" s="3" t="inlineStr">
         <is>
           <t>VWM - Summer Women's Mix</t>
         </is>
       </c>
-      <c r="G2" s="3" t="n">
+      <c r="H2" s="4" t="n">
         <v>9.99</v>
       </c>
-      <c r="H2" s="4" t="n">
+      <c r="I2" s="5" t="n">
         <v>46248</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>Ralph Lauren Polo</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="C3" s="3" t="inlineStr">
         <is>
           <t>Navy with pinstripes</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr"/>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="D3" s="3" t="inlineStr"/>
+      <c r="E3" s="3" t="inlineStr">
         <is>
           <t>XXL</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="F3" s="3" t="inlineStr">
         <is>
           <t>Very good vintage condition</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr"/>
-      <c r="G3" s="3" t="n">
+      <c r="G3" s="3" t="inlineStr"/>
+      <c r="H3" s="4" t="n">
         <v>14.99</v>
       </c>
-      <c r="H3" s="4" t="n">
+      <c r="I3" s="5" t="n">
         <v>46248</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>Ralph Lauren Polo</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="C4" s="3" t="inlineStr">
         <is>
           <t>Tartan check, labels cut</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr"/>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="D4" s="3" t="inlineStr"/>
+      <c r="E4" s="3" t="inlineStr">
         <is>
           <t>Small Men's</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="F4" s="3" t="inlineStr">
         <is>
           <t>Very good condition</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="G4" s="3" t="inlineStr">
         <is>
           <t>VWM - RL Lacoste Polos</t>
         </is>
       </c>
-      <c r="G4" s="3" t="n">
+      <c r="H4" s="4" t="n">
         <v>14.99</v>
       </c>
-      <c r="H4" s="4" t="n">
+      <c r="I4" s="5" t="n">
         <v>46248</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+      <c r="A5" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>Ralph Lauren Women's Polo Shirt</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="C5" s="3" t="inlineStr">
         <is>
           <t>Black</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr"/>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="D5" s="3" t="inlineStr"/>
+      <c r="E5" s="3" t="inlineStr">
         <is>
           <t>Large Women's</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr">
+      <c r="F5" s="3" t="inlineStr">
         <is>
           <t>Very good condition</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr">
+      <c r="G5" s="3" t="inlineStr">
         <is>
           <t>VWM - Women's Y2K Mix</t>
         </is>
       </c>
-      <c r="G5" s="3" t="n">
+      <c r="H5" s="4" t="n">
         <v>12.99</v>
       </c>
-      <c r="H5" s="4" t="n">
+      <c r="I5" s="5" t="n">
         <v>46248</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="A6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
         <is>
           <t>Women's Bralette</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="C6" s="3" t="inlineStr">
         <is>
           <t>Red</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="D6" s="3" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="E6" s="3" t="inlineStr">
         <is>
           <t>36</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="F6" s="3" t="inlineStr">
         <is>
           <t>Very good condition</t>
         </is>
       </c>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="G6" s="3" t="inlineStr">
         <is>
           <t>VWM - Women's Summer Mix</t>
         </is>
       </c>
-      <c r="G6" s="3" t="n">
+      <c r="H6" s="4" t="n">
         <v>12.99</v>
       </c>
-      <c r="H6" s="4" t="n">
+      <c r="I6" s="5" t="n">
         <v>46248</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+      <c r="A7" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>Women's Bralette</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="C7" s="3" t="inlineStr">
         <is>
           <t>Black</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="D7" s="3" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="E7" s="3" t="inlineStr">
         <is>
           <t>Small</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr">
+      <c r="F7" s="3" t="inlineStr">
         <is>
           <t>Very good condition</t>
         </is>
       </c>
-      <c r="F7" s="2" t="inlineStr">
+      <c r="G7" s="3" t="inlineStr">
         <is>
           <t>VWM - Women's Y2K Mix</t>
         </is>
       </c>
-      <c r="G7" s="3" t="n">
+      <c r="H7" s="4" t="n">
         <v>8.99</v>
       </c>
-      <c r="H7" s="4" t="n">
+      <c r="I7" s="5" t="n">
         <v>46248</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+      <c r="A8" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t>Ralph Lauren Women's Polo</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="C8" s="3" t="inlineStr">
         <is>
           <t>Navy</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr"/>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="D8" s="3" t="inlineStr"/>
+      <c r="E8" s="3" t="inlineStr">
         <is>
           <t>Medium (10-12)</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr">
+      <c r="F8" s="3" t="inlineStr">
         <is>
           <t>Very good condition</t>
         </is>
       </c>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="G8" s="3" t="inlineStr">
         <is>
           <t>VWM - Women's Y2K Mix</t>
         </is>
       </c>
-      <c r="G8" s="3" t="inlineStr"/>
       <c r="H8" s="4" t="n">
+        <v>12.99</v>
+      </c>
+      <c r="I8" s="5" t="n">
         <v>46248</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+      <c r="A9" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
         <is>
           <t>Nike Track Jacket</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="C9" s="3" t="inlineStr">
         <is>
           <t>Green</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr"/>
-      <c r="D9" s="2" t="inlineStr">
+      <c r="D9" s="3" t="inlineStr"/>
+      <c r="E9" s="3" t="inlineStr">
         <is>
           <t>Large (oversized fit)</t>
         </is>
       </c>
-      <c r="E9" s="2" t="inlineStr">
+      <c r="F9" s="3" t="inlineStr">
         <is>
           <t>Very good condition</t>
         </is>
       </c>
-      <c r="F9" s="2" t="inlineStr">
+      <c r="G9" s="3" t="inlineStr">
         <is>
           <t>VWM - Track Jacket</t>
         </is>
       </c>
-      <c r="G9" s="3" t="n">
+      <c r="H9" s="4" t="n">
         <v>24.99</v>
       </c>
-      <c r="H9" s="4" t="n">
+      <c r="I9" s="5" t="n">
         <v>46248</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+      <c r="A10" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
         <is>
           <t>Harley Davidson Women's Cardigan</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="C10" s="3" t="inlineStr">
         <is>
           <t>White</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="D10" s="3" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr"/>
-      <c r="E10" s="2" t="inlineStr">
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
         <is>
           <t>Very good condition</t>
         </is>
       </c>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="G10" s="3" t="inlineStr">
         <is>
           <t>VWM - Women's Y2K Mix</t>
         </is>
       </c>
-      <c r="G10" s="3" t="n">
+      <c r="H10" s="4" t="n">
         <v>14.99</v>
       </c>
-      <c r="H10" s="4" t="n">
+      <c r="I10" s="5" t="n">
         <v>46248</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+      <c r="A11" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
         <is>
           <t>Ralph Lauren Women's Polo</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr">
+      <c r="C11" s="3" t="inlineStr">
         <is>
           <t>Navy</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="D11" s="3" t="inlineStr">
         <is>
           <t>One small discrepancy on the front (see images)</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="E11" s="3" t="inlineStr">
         <is>
           <t>XL Women's</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="F11" s="3" t="inlineStr">
         <is>
           <t>Very good vintage condition</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="G11" s="3" t="inlineStr">
         <is>
           <t>VWM - RL Lacoste Polos</t>
         </is>
       </c>
-      <c r="G11" s="3" t="n">
+      <c r="H11" s="4" t="n">
         <v>9.99</v>
       </c>
-      <c r="H11" s="4" t="n">
+      <c r="I11" s="5" t="n">
         <v>46248</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+      <c r="A12" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
         <is>
           <t>Nike Track Jacket</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="C12" s="3" t="inlineStr">
         <is>
           <t>Black and navy</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr">
+      <c r="D12" s="3" t="inlineStr">
         <is>
           <t>White marks on right sleeve (see images)</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
+      <c r="E12" s="3" t="inlineStr">
         <is>
           <t>XL</t>
         </is>
       </c>
-      <c r="E12" s="2" t="inlineStr">
+      <c r="F12" s="3" t="inlineStr">
         <is>
           <t>Very good vintage condition</t>
         </is>
       </c>
-      <c r="F12" s="2" t="inlineStr">
+      <c r="G12" s="3" t="inlineStr">
         <is>
           <t>VWM - Track Jacket</t>
         </is>
       </c>
-      <c r="G12" s="3" t="inlineStr"/>
       <c r="H12" s="4" t="n">
+        <v>14.99</v>
+      </c>
+      <c r="I12" s="5" t="n">
         <v>46248</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="inlineStr">
+      <c r="A13" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
         <is>
           <t>Ralph Lauren Polo</t>
         </is>
       </c>
-      <c r="B13" s="2" t="inlineStr">
+      <c r="C13" s="3" t="inlineStr">
         <is>
           <t>Green with orange pony</t>
         </is>
       </c>
-      <c r="C13" s="2" t="inlineStr">
+      <c r="D13" s="3" t="inlineStr">
         <is>
           <t>Discrepancies on the front</t>
         </is>
       </c>
-      <c r="D13" s="2" t="inlineStr">
+      <c r="E13" s="3" t="inlineStr">
         <is>
           <t>XXL Men's</t>
         </is>
       </c>
-      <c r="E13" s="2" t="inlineStr">
+      <c r="F13" s="3" t="inlineStr">
         <is>
           <t>Good condition</t>
         </is>
       </c>
-      <c r="F13" s="2" t="inlineStr">
+      <c r="G13" s="3" t="inlineStr">
         <is>
           <t>VWM - RL Lacoste Polos</t>
         </is>
       </c>
-      <c r="G13" s="3" t="n">
+      <c r="H13" s="4" t="n">
         <v>9.99</v>
       </c>
-      <c r="H13" s="4" t="n">
+      <c r="I13" s="5" t="n">
         <v>46248</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="inlineStr">
+      <c r="A14" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
         <is>
           <t>Lacoste Polo</t>
         </is>
       </c>
-      <c r="B14" s="2" t="inlineStr">
+      <c r="C14" s="3" t="inlineStr">
         <is>
           <t>Light green</t>
         </is>
       </c>
-      <c r="C14" s="2" t="inlineStr">
+      <c r="D14" s="3" t="inlineStr">
         <is>
           <t>Discrepancies on the front (see images)</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr">
+      <c r="E14" s="3" t="inlineStr">
         <is>
           <t>UK Small</t>
         </is>
       </c>
-      <c r="E14" s="2" t="inlineStr">
+      <c r="F14" s="3" t="inlineStr">
         <is>
           <t>Good condition</t>
         </is>
       </c>
-      <c r="F14" s="2" t="inlineStr">
+      <c r="G14" s="3" t="inlineStr">
         <is>
           <t>VWM - RL Lacoste Polos</t>
         </is>
       </c>
-      <c r="G14" s="3" t="n">
+      <c r="H14" s="4" t="n">
         <v>9.99</v>
       </c>
-      <c r="H14" s="4" t="n">
+      <c r="I14" s="5" t="n">
         <v>46248</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="inlineStr">
+      <c r="A15" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
         <is>
           <t>Lacoste Polo</t>
         </is>
       </c>
-      <c r="B15" s="2" t="inlineStr">
+      <c r="C15" s="3" t="inlineStr">
         <is>
           <t>Dark green</t>
         </is>
       </c>
-      <c r="C15" s="2" t="inlineStr">
+      <c r="D15" s="3" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="D15" s="2" t="inlineStr">
+      <c r="E15" s="3" t="inlineStr">
         <is>
           <t>UK Large</t>
         </is>
       </c>
-      <c r="E15" s="2" t="inlineStr">
+      <c r="F15" s="3" t="inlineStr">
         <is>
           <t>Very good vintage condition</t>
         </is>
       </c>
-      <c r="F15" s="2" t="inlineStr">
+      <c r="G15" s="3" t="inlineStr">
         <is>
           <t>VWM - RL Lacoste Polos</t>
         </is>
       </c>
-      <c r="G15" s="3" t="n">
+      <c r="H15" s="4" t="n">
+        <v>12.99</v>
+      </c>
+      <c r="I15" s="5" t="n">
+        <v>46248</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>Ralph Lauren Polo</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>Turquoise</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr"/>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>Large</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>Very good condition</t>
+        </is>
+      </c>
+      <c r="G16" s="3" t="inlineStr">
+        <is>
+          <t>VWM - RL Lacoste Polos</t>
+        </is>
+      </c>
+      <c r="H16" s="4" t="n">
         <v>14.99</v>
       </c>
-      <c r="H15" s="4" t="n">
-        <v>46248</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>Ralph Lauren Polo</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>Turquoise</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="inlineStr"/>
-      <c r="D16" s="2" t="inlineStr">
-        <is>
-          <t>Large</t>
-        </is>
-      </c>
-      <c r="E16" s="2" t="inlineStr">
-        <is>
-          <t>Very good condition</t>
-        </is>
-      </c>
-      <c r="F16" s="2" t="inlineStr">
-        <is>
-          <t>VWM - RL Lacoste Polos</t>
-        </is>
-      </c>
-      <c r="G16" s="3" t="n">
-        <v>14.99</v>
-      </c>
-      <c r="H16" s="4" t="n">
+      <c r="I16" s="5" t="n">
         <v>46248</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H16"/>
+  <autoFilter ref="A1:I16"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>